<commit_message>
DOI units (NPS, USFWS, BLM, BIA) relabeled WFS (Wildland Fire Service) in FDRA titles and agency; 80th/95th standard now set by the standard_90_97 field
</commit_message>
<xml_diff>
--- a/site/thresholds/FDRA_thresholds.xlsx
+++ b/site/thresholds/FDRA_thresholds.xlsx
@@ -18487,7 +18487,7 @@
       <c r="P14" s="4" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BDU "Desert FDRA" from the unit survey: BI-X dispatch Low 0-25, Moderate to 50, High above. Stations 45112, 45134. </t>
+          <t>CAL FIRE BDU "Desert FDRA" from the unit survey: BI-X dispatch Low 0-25, Moderate to 50, High above. Stations 45112, 45134.</t>
         </is>
       </c>
     </row>
@@ -18542,7 +18542,7 @@
       <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BDU "Mountain FDRA" from the unit survey: BI-Y dispatch Low 0-10, Moderate to 25, High above. Stations 45101, 45133. </t>
+          <t>CAL FIRE BDU "Mountain FDRA" from the unit survey: BI-Y dispatch Low 0-10, Moderate to 25, High above. Stations 45101, 45133.</t>
         </is>
       </c>
     </row>
@@ -18683,7 +18683,7 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BDU "Valley FDRA" from the unit survey: BI-X dispatch Low 0-25, Moderate to 79, High above. Stations 45113, 480306, 45114. </t>
+          <t>CAL FIRE BDU "Valley FDRA" from the unit survey: BI-X dispatch Low 0-25, Moderate to 79, High above. Stations 45113, 480306, 45114.</t>
         </is>
       </c>
     </row>
@@ -18738,7 +18738,7 @@
       <c r="P19" s="4" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BEU "Salinas Valley Grass FDRA" from the unit survey: BI-X dispatch Low 0-196, Moderate to 252, High above. Stations 44303, 44310. </t>
+          <t>CAL FIRE BEU "Salinas Valley Grass FDRA" from the unit survey: BI-X dispatch Low 0-196, Moderate to 252, High above. Stations 44303, 44310.</t>
         </is>
       </c>
     </row>
@@ -18793,7 +18793,7 @@
       <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BEU "Gabilan FDRA" from the unit survey: BI-X dispatch Low 0-144, Moderate to 209, High above. Stations 44310, 44410, 44409. </t>
+          <t>CAL FIRE BEU "Gabilan FDRA" from the unit survey: BI-X dispatch Low 0-144, Moderate to 209, High above. Stations 44310, 44410, 44409.</t>
         </is>
       </c>
     </row>
@@ -18848,7 +18848,7 @@
       <c r="P21" s="4" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BEU "Coastal Timber FDRA" from the unit survey: BI-W dispatch Low 0-22, Moderate to 38, High above. Stations 44301, 44302. </t>
+          <t>CAL FIRE BEU "Coastal Timber FDRA" from the unit survey: BI-W dispatch Low 0-22, Moderate to 38, High above. Stations 44301, 44302.</t>
         </is>
       </c>
     </row>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>BLM</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -18928,7 +18928,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>BLM</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -18991,7 +18991,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>BLM</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -19054,7 +19054,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -19085,7 +19085,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>BLM</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -19136,7 +19136,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>BLM</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -19256,7 +19256,7 @@
       <c r="P29" s="4" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BTU "Foothill" from the unit survey: BI-X dispatch Low 0-54, Moderate to 140, High above. Stations 41211, 41214, 40805. </t>
+          <t>CAL FIRE BTU "Foothill" from the unit survey: BI-X dispatch Low 0-54, Moderate to 140, High above. Stations 41211, 41214, 40805.</t>
         </is>
       </c>
     </row>
@@ -19311,7 +19311,7 @@
       <c r="P30" s="4" t="inlineStr"/>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BTU "Valley" from the unit survey: BI-W dispatch Low 0-10, Moderate to 28, High above. Stations 41201, 40814, 41215. </t>
+          <t>CAL FIRE BTU "Valley" from the unit survey: BI-W dispatch Low 0-10, Moderate to 28, High above. Stations 41201, 40814, 41215.</t>
         </is>
       </c>
     </row>
@@ -19366,7 +19366,7 @@
       <c r="P31" s="4" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE BTU "Mountain" from the unit survey: BI-Z dispatch Low 0-30, Moderate to 72, High above. Stations 41213, 41701, 41214. </t>
+          <t>CAL FIRE BTU "Mountain" from the unit survey: BI-Z dispatch Low 0-30, Moderate to 72, High above. Stations 41213, 41701, 41214.</t>
         </is>
       </c>
     </row>
@@ -19383,7 +19383,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>BLM / NPS (CDIFP)</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -19442,7 +19442,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>BLM / NPS (CDIFP)</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -19501,7 +19501,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>BLM / NPS (CDIFP)</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -19560,7 +19560,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>BLM / NPS (CDIFP)</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -19854,7 +19854,7 @@
       <c r="P39" s="4" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE CZU "Coast FDRA" from the unit survey: BI-Y dispatch Low 0-13, Moderate to 22, High above. Stations 43802, 43304. </t>
+          <t>CAL FIRE CZU "Coast FDRA" from the unit survey: BI-Y dispatch Low 0-13, Moderate to 22, High above. Stations 43802, 43304.</t>
         </is>
       </c>
     </row>
@@ -19909,7 +19909,7 @@
       <c r="P40" s="4" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE CZU "Inland FDRA" from the unit survey: BI-Z dispatch Low 0-55.9, Moderate to 75, High above. Stations 43809, 43404. </t>
+          <t>CAL FIRE CZU "Inland FDRA" from the unit survey: BI-Z dispatch Low 0-55.9, Moderate to 75, High above. Stations 43809, 43404.</t>
         </is>
       </c>
     </row>
@@ -20286,7 +20286,7 @@
       <c r="P47" s="4" t="inlineStr"/>
       <c r="Q47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE HUU "Alderpoint" from the unit survey: BI-Y dispatch Low 0-15.9, Moderate to 18.9, High above. Stations 40423. </t>
+          <t>CAL FIRE HUU "Alderpoint" from the unit survey: BI-Y dispatch Low 0-15.9, Moderate to 18.9, High above. Stations 40423.</t>
         </is>
       </c>
     </row>
@@ -20341,7 +20341,7 @@
       <c r="P48" s="4" t="inlineStr"/>
       <c r="Q48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE HUU "Coastal Strip" from the unit survey: BI-Y dispatch Low 0-16.9, Moderate to 21.9, High above. Stations 40429. </t>
+          <t>CAL FIRE HUU "Coastal Strip" from the unit survey: BI-Y dispatch Low 0-16.9, Moderate to 21.9, High above. Stations 40429.</t>
         </is>
       </c>
     </row>
@@ -20396,7 +20396,7 @@
       <c r="P49" s="4" t="inlineStr"/>
       <c r="Q49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE HUU "Eel River" from the unit survey: BI-Y dispatch Low 0-17.9, Moderate to 22.9, High above. Stations 40421. </t>
+          <t>CAL FIRE HUU "Eel River" from the unit survey: BI-Y dispatch Low 0-17.9, Moderate to 22.9, High above. Stations 40421.</t>
         </is>
       </c>
     </row>
@@ -21264,7 +21264,7 @@
       <c r="P65" s="4" t="inlineStr"/>
       <c r="Q65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LMU "LMU NE" from the unit survey: BI-X dispatch Low 0-125, Moderate to 210, High above. Stations 40308, 40309. </t>
+          <t>CAL FIRE LMU "LMU NE" from the unit survey: BI-X dispatch Low 0-125, Moderate to 210, High above. Stations 40308, 40309.</t>
         </is>
       </c>
     </row>
@@ -21319,7 +21319,7 @@
       <c r="P66" s="4" t="inlineStr"/>
       <c r="Q66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LMU "LMU NW" from the unit survey: BI-X dispatch Low 0-50, Moderate to 171, High above. Stations 40221, 40312. </t>
+          <t>CAL FIRE LMU "LMU NW" from the unit survey: BI-X dispatch Low 0-50, Moderate to 171, High above. Stations 40221, 40312.</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       <c r="P67" s="4" t="inlineStr"/>
       <c r="Q67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LMU "LMU SE" from the unit survey: BI-X dispatch Low 0-92, Moderate to 162, High above. Stations 40709, 40721, 40732. </t>
+          <t>CAL FIRE LMU "LMU SE" from the unit survey: BI-X dispatch Low 0-92, Moderate to 162, High above. Stations 40709, 40721, 40732.</t>
         </is>
       </c>
     </row>
@@ -21429,7 +21429,7 @@
       <c r="P68" s="4" t="inlineStr"/>
       <c r="Q68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LMU "LMU SW" from the unit survey: BI-X dispatch Low 0-65, Moderate to 165, High above. Stations 40719, 40904. </t>
+          <t>CAL FIRE LMU "LMU SW" from the unit survey: BI-X dispatch Low 0-65, Moderate to 165, High above. Stations 40719, 40904.</t>
         </is>
       </c>
     </row>
@@ -21688,7 +21688,7 @@
       <c r="P73" s="4" t="inlineStr"/>
       <c r="Q73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LNU "Central" from the unit survey: BI-W dispatch Low 0-25, Moderate to 45, High above. Stations 41409. </t>
+          <t>CAL FIRE LNU "Central" from the unit survey: BI-W dispatch Low 0-25, Moderate to 45, High above. Stations 41409.</t>
         </is>
       </c>
     </row>
@@ -21743,7 +21743,7 @@
       <c r="P74" s="4" t="inlineStr"/>
       <c r="Q74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LNU "Eastside" from the unit survey: BI-V dispatch Low 0-33, Moderate to 51, High above. Stations 42202. </t>
+          <t>CAL FIRE LNU "Eastside" from the unit survey: BI-V dispatch Low 0-33, Moderate to 51, High above. Stations 42202.</t>
         </is>
       </c>
     </row>
@@ -21798,7 +21798,7 @@
       <c r="P75" s="4" t="inlineStr"/>
       <c r="Q75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LNU "Mayacamas" from the unit survey: BI-V dispatch Low 0-29, Moderate to 55, High above. Stations 42010. </t>
+          <t>CAL FIRE LNU "Mayacamas" from the unit survey: BI-V dispatch Low 0-29, Moderate to 55, High above. Stations 42010.</t>
         </is>
       </c>
     </row>
@@ -21853,7 +21853,7 @@
       <c r="P76" s="4" t="inlineStr"/>
       <c r="Q76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LNU "Southend" from the unit survey: BI-V dispatch Low 0-34, Moderate to 43, High above. Stations 42310. </t>
+          <t>CAL FIRE LNU "Southend" from the unit survey: BI-V dispatch Low 0-34, Moderate to 43, High above. Stations 42310.</t>
         </is>
       </c>
     </row>
@@ -21939,7 +21939,7 @@
       <c r="P78" s="4" t="inlineStr"/>
       <c r="Q78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE LNU "Westside" from the unit survey: BI-W dispatch Low 0-24, Moderate to 40, High above. Stations 42009. </t>
+          <t>CAL FIRE LNU "Westside" from the unit survey: BI-W dispatch Low 0-24, Moderate to 40, High above. Stations 42009.</t>
         </is>
       </c>
     </row>
@@ -23828,7 +23828,7 @@
       <c r="P117" s="4" t="inlineStr"/>
       <c r="Q117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE NEU "Placer FDRA" from the unit survey: BI-W dispatch Low 0-10, Moderate to 30, High above. Stations 41907, 42609. </t>
+          <t>CAL FIRE NEU "Placer FDRA" from the unit survey: BI-W dispatch Low 0-10, Moderate to 30, High above. Stations 41907, 42609.</t>
         </is>
       </c>
     </row>
@@ -23914,7 +23914,7 @@
       <c r="P119" s="4" t="inlineStr"/>
       <c r="Q119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE NEU "Western FDRA" from the unit survey: BI-W dispatch Low 0-10, Moderate to 30, High above. Stations 41201, 42609, 41907. </t>
+          <t>CAL FIRE NEU "Western FDRA" from the unit survey: BI-W dispatch Low 0-10, Moderate to 30, High above. Stations 41201, 42609, 41907.</t>
         </is>
       </c>
     </row>
@@ -23931,7 +23931,7 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -23978,7 +23978,7 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr"/>
@@ -24009,7 +24009,7 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -24056,7 +24056,7 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -24111,7 +24111,7 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
@@ -24166,7 +24166,7 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -24221,7 +24221,7 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
@@ -24276,7 +24276,7 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -24323,7 +24323,7 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -24390,7 +24390,7 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -24457,7 +24457,7 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -24524,7 +24524,7 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
@@ -24638,7 +24638,7 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -24705,7 +24705,7 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -24772,7 +24772,7 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -25498,7 +25498,7 @@
       <c r="P151" s="4" t="inlineStr"/>
       <c r="Q151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SCU "South FDRA" from the unit survey: BI-Y dispatch Low 0-16.9, Moderate to 20.9, High above. Stations 43913, 43912. </t>
+          <t>CAL FIRE SCU "South FDRA" from the unit survey: BI-Y dispatch Low 0-16.9, Moderate to 20.9, High above. Stations 43913, 43912.</t>
         </is>
       </c>
     </row>
@@ -25553,7 +25553,7 @@
       <c r="P152" s="4" t="inlineStr"/>
       <c r="Q152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SCU "Central FDRA" from the unit survey: BI-Y dispatch Low 0-21.9, Moderate to 30.9, High above. Stations 43502, 43404. </t>
+          <t>CAL FIRE SCU "Central FDRA" from the unit survey: BI-Y dispatch Low 0-21.9, Moderate to 30.9, High above. Stations 43502, 43404.</t>
         </is>
       </c>
     </row>
@@ -25663,7 +25663,7 @@
       <c r="P154" s="4" t="inlineStr"/>
       <c r="Q154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SCU "Northeast FDRA" from the unit survey: BI-Y dispatch Low 0-23.9, Moderate to 33.9, High above. Stations 43008, 43011, 43013, 43407. </t>
+          <t>CAL FIRE SCU "Northeast FDRA" from the unit survey: BI-Y dispatch Low 0-23.9, Moderate to 33.9, High above. Stations 43008, 43011, 43013, 43407.</t>
         </is>
       </c>
     </row>
@@ -26623,7 +26623,7 @@
       <c r="P170" s="4" t="inlineStr"/>
       <c r="Q170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SLU "Coastal FDRA" from the unit survey: BI-Y dispatch Low 0-11, Moderate to 17, High above. Stations 44917. </t>
+          <t>CAL FIRE SLU "Coastal FDRA" from the unit survey: BI-Y dispatch Low 0-11, Moderate to 17, High above. Stations 44917.</t>
         </is>
       </c>
     </row>
@@ -26678,7 +26678,7 @@
       <c r="P171" s="4" t="inlineStr"/>
       <c r="Q171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SLU "Coastal Valley FDRA" from the unit survey: BI-Y dispatch Low 0-12, Moderate to 21, High above. Stations 44915. </t>
+          <t>CAL FIRE SLU "Coastal Valley FDRA" from the unit survey: BI-Y dispatch Low 0-12, Moderate to 21, High above. Stations 44915.</t>
         </is>
       </c>
     </row>
@@ -26733,7 +26733,7 @@
       <c r="P172" s="4" t="inlineStr"/>
       <c r="Q172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE SLU "Inland Grass FDRA" from the unit survey: BI-Y dispatch Low 0-16, Moderate to 31, High above. Stations 44914. </t>
+          <t>CAL FIRE SLU "Inland Grass FDRA" from the unit survey: BI-Y dispatch Low 0-16, Moderate to 31, High above. Stations 44914.</t>
         </is>
       </c>
     </row>
@@ -27677,7 +27677,7 @@
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>USFS / WFS</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
@@ -27965,7 +27965,7 @@
       <c r="P194" s="4" t="inlineStr"/>
       <c r="Q194" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TCU "Foothills West" from the unit survey: IC-Y dispatch Low 0-16, Moderate to 29, High above. Stations 43613. </t>
+          <t>CAL FIRE TCU "Foothills West" from the unit survey: IC-Y dispatch Low 0-16, Moderate to 29, High above. Stations 43613.</t>
         </is>
       </c>
     </row>
@@ -28113,7 +28113,7 @@
       <c r="P198" s="4" t="inlineStr"/>
       <c r="Q198" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TGU "Timber" from the unit survey: BI-Y dispatch Low 0-12, Moderate to 27, High above. Stations 40815, 40805, 40801. </t>
+          <t>CAL FIRE TGU "Timber" from the unit survey: BI-Y dispatch Low 0-12, Moderate to 27, High above. Stations 40815, 40805, 40801.</t>
         </is>
       </c>
     </row>
@@ -28168,7 +28168,7 @@
       <c r="P199" s="4" t="inlineStr"/>
       <c r="Q199" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TGU "Grass" from the unit survey: SC-V dispatch Low 0-10, Moderate to 90, High above. Stations 40814, 41215. </t>
+          <t>CAL FIRE TGU "Grass" from the unit survey: SC-V dispatch Low 0-10, Moderate to 90, High above. Stations 40814, 41215.</t>
         </is>
       </c>
     </row>
@@ -28223,7 +28223,7 @@
       <c r="P200" s="4" t="inlineStr"/>
       <c r="Q200" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TGU "Brush" from the unit survey: BI-W dispatch Low 0-12, Moderate to 50, High above. Stations 40816, 40802. </t>
+          <t>CAL FIRE TGU "Brush" from the unit survey: BI-W dispatch Low 0-12, Moderate to 50, High above. Stations 40816, 40802.</t>
         </is>
       </c>
     </row>
@@ -28337,7 +28337,7 @@
       <c r="P202" s="4" t="inlineStr"/>
       <c r="Q202" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TUU "TUU" from the unit survey: BI-X dispatch Low 0-89, Moderate to 144, High above. Stations 44731, 44708. </t>
+          <t>CAL FIRE TUU "TUU" from the unit survey: BI-X dispatch Low 0-89, Moderate to 144, High above. Stations 44731, 44708.</t>
         </is>
       </c>
     </row>
@@ -28349,12 +28349,12 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>Bia</t>
+          <t>Tule River Reservation (WFS)</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr"/>
@@ -28454,7 +28454,7 @@
       <c r="P205" s="4" t="inlineStr"/>
       <c r="Q205" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAL FIRE TUU "TUU" from the unit survey: BI-X dispatch Low 0-89, Moderate to 144, High above. Stations 44731, 44708. </t>
+          <t>CAL FIRE TUU "TUU" from the unit survey: BI-X dispatch Low 0-89, Moderate to 144, High above. Stations 44731, 44708.</t>
         </is>
       </c>
     </row>
@@ -28471,7 +28471,7 @@
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr"/>
@@ -28502,7 +28502,7 @@
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr"/>
@@ -28533,7 +28533,7 @@
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr"/>
@@ -28564,7 +28564,7 @@
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
@@ -28615,7 +28615,7 @@
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
@@ -28662,7 +28662,7 @@
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D211" s="4" t="inlineStr">
@@ -28717,7 +28717,7 @@
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
@@ -28772,7 +28772,7 @@
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
@@ -28827,7 +28827,7 @@
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
@@ -28874,7 +28874,7 @@
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>USFWS</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
@@ -28920,12 +28920,12 @@
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>Ufw-Lkr</t>
+          <t>Lkr</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>CAL FIRE / interagency</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Area settings (docs/assets/area.js) replace California hardcodes; decision tools gain matrices, multi-day windows and one-class adjustments (workbook + popups); SC values carried into popups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016iZr4gXkGeU9qaRaPUJHXS
</commit_message>
<xml_diff>
--- a/site/thresholds/FDRA_thresholds.xlsx
+++ b/site/thresholds/FDRA_thresholds.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to update" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thresholds" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FDOP info" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrix tools" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FDOP info" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -506,75 +507,131 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - FDOP info sheet: one row per FDRA (the plan source, SIG stations, season and so on).</t>
+          <t xml:space="preserve">     Days used (optional): which days the tool averages. Blank = the observed day and the forecast day.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Rows with no FDOP source and no tools are ignored.</t>
+          <t xml:space="preserve">     F1 = the next forecast day only; O1+F1+F2+F3 = average of yesterday's observed and the next three forecast days.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - To change a threshold, edit its row. To add a tool, add a row with the FDRA ID.</t>
+          <t xml:space="preserve">     Adjustments (optional): move the class up or down when a condition is met, one per line or separated by ;</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     To remove a tool, delete the row.</t>
+          <t xml:space="preserve">     for example  Tmax &lt; 57 : -1   or   GSI &gt; 0.3 : -1   or   100-hr FM &gt; 14 : -1 @F1  (the @ part sets its own days).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3. Upload it to GitHub: open the site/thresholds folder, then Add file, then Upload files. Drop the</t>
+          <t xml:space="preserve">     Variables: Tmax, RH min, 100-hr FM, 1000-hr FM, GSI, KBDI, ERC, BI, IC, SC.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   file in, write a short note (for example "LPF 2027 FDOP"), and Commit changes.</t>
+          <t xml:space="preserve">   - Matrix tools sheet: a level read from a table, such as BI rows x ERC columns. Give the row index and</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4. The "Thresholds check" run starts on its own. A green check means the file is good. A red X lists</t>
+          <t xml:space="preserve">     breakpoints, the column index and breakpoints, then one "Row N levels" cell per row with the level for each</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   each problem by sheet and row. Fix those rows and upload again. FDRAs with errors keep their last</t>
+          <t xml:space="preserve">     column, separated by spaces (for example 1 1 1 2 3). Levels are numbers from 1 to the number of classes.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   good values; everything else updates.</t>
+          <t xml:space="preserve">   - FDOP info sheet: one row per FDRA (the plan source, SIG stations, season and so on).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>5. The site and the AGOL popups pick up the new thresholds at the next site build, which starts on</t>
+          <t xml:space="preserve">     Rows with no FDOP source and no tools are ignored.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - To change a threshold, edit its row. To add a tool, add a row with the FDRA ID.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     To remove a tool, delete the row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>3. Upload it to GitHub: open the site/thresholds folder, then Add file, then Upload files. Drop the</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   file in, write a short note (for example "LPF 2027 FDOP"), and Commit changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>4. The "Thresholds check" run starts on its own. A green check means the file is good. A red X lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   each problem by sheet and row. Fix those rows and upload again. FDRAs with errors keep their last</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   good values; everything else updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>5. The site and the AGOL popups pick up the new thresholds at the next site build, which starts on</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   its own after the upload (about 15-30 minutes).</t>
         </is>
@@ -591,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R298"/>
+  <dimension ref="A1:T298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -612,6 +669,8 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,6 +764,16 @@
           <t>Class 7</t>
         </is>
       </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Days used</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Adjustments</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -755,6 +824,8 @@
       <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="n"/>
       <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -819,6 +890,8 @@
       </c>
       <c r="Q3" s="4" t="n"/>
       <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -883,6 +956,8 @@
       </c>
       <c r="Q4" s="4" t="n"/>
       <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -947,6 +1022,8 @@
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="inlineStr"/>
+      <c r="T5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1011,6 +1088,8 @@
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1075,6 +1154,8 @@
       </c>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
+      <c r="S7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1139,6 +1220,8 @@
       </c>
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1203,6 +1286,8 @@
       </c>
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1260,6 +1345,8 @@
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1324,6 +1411,8 @@
       </c>
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="inlineStr"/>
+      <c r="T11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1388,6 +1477,8 @@
       </c>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1452,6 +1543,8 @@
       </c>
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1509,6 +1602,8 @@
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1573,6 +1668,8 @@
       </c>
       <c r="Q15" s="4" t="n"/>
       <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1637,6 +1734,8 @@
       </c>
       <c r="Q16" s="4" t="n"/>
       <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1701,6 +1800,8 @@
       </c>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1758,6 +1859,8 @@
       <c r="P18" s="4" t="n"/>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1822,6 +1925,8 @@
       </c>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1886,6 +1991,8 @@
       </c>
       <c r="Q20" s="4" t="n"/>
       <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1950,6 +2057,8 @@
       </c>
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="inlineStr"/>
+      <c r="T21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2007,6 +2116,8 @@
       <c r="P22" s="4" t="n"/>
       <c r="Q22" s="4" t="n"/>
       <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2071,6 +2182,8 @@
       </c>
       <c r="Q23" s="4" t="n"/>
       <c r="R23" s="4" t="n"/>
+      <c r="S23" s="4" t="inlineStr"/>
+      <c r="T23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2135,6 +2248,8 @@
       </c>
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2199,6 +2314,8 @@
       </c>
       <c r="Q25" s="4" t="n"/>
       <c r="R25" s="4" t="n"/>
+      <c r="S25" s="4" t="inlineStr"/>
+      <c r="T25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2256,6 +2373,8 @@
       <c r="P26" s="4" t="n"/>
       <c r="Q26" s="4" t="n"/>
       <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="inlineStr"/>
+      <c r="T26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2320,6 +2439,8 @@
       </c>
       <c r="Q27" s="4" t="n"/>
       <c r="R27" s="4" t="n"/>
+      <c r="S27" s="4" t="inlineStr"/>
+      <c r="T27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2384,6 +2505,8 @@
       </c>
       <c r="Q28" s="4" t="n"/>
       <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="inlineStr"/>
+      <c r="T28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2434,6 +2557,8 @@
       <c r="P29" s="4" t="n"/>
       <c r="Q29" s="4" t="n"/>
       <c r="R29" s="4" t="n"/>
+      <c r="S29" s="4" t="inlineStr"/>
+      <c r="T29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2484,6 +2609,8 @@
       <c r="P30" s="4" t="n"/>
       <c r="Q30" s="4" t="n"/>
       <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="inlineStr"/>
+      <c r="T30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2534,6 +2661,8 @@
       <c r="P31" s="4" t="n"/>
       <c r="Q31" s="4" t="n"/>
       <c r="R31" s="4" t="n"/>
+      <c r="S31" s="4" t="inlineStr"/>
+      <c r="T31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2584,6 +2713,8 @@
       <c r="P32" s="4" t="n"/>
       <c r="Q32" s="4" t="n"/>
       <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="inlineStr"/>
+      <c r="T32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2634,6 +2765,8 @@
       <c r="P33" s="4" t="n"/>
       <c r="Q33" s="4" t="n"/>
       <c r="R33" s="4" t="n"/>
+      <c r="S33" s="4" t="inlineStr"/>
+      <c r="T33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2684,6 +2817,8 @@
       <c r="P34" s="4" t="n"/>
       <c r="Q34" s="4" t="n"/>
       <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="inlineStr"/>
+      <c r="T34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2734,6 +2869,8 @@
       <c r="P35" s="4" t="n"/>
       <c r="Q35" s="4" t="n"/>
       <c r="R35" s="4" t="n"/>
+      <c r="S35" s="4" t="inlineStr"/>
+      <c r="T35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2784,6 +2921,8 @@
       <c r="P36" s="4" t="n"/>
       <c r="Q36" s="4" t="n"/>
       <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="inlineStr"/>
+      <c r="T36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2834,6 +2973,8 @@
       <c r="P37" s="4" t="n"/>
       <c r="Q37" s="4" t="n"/>
       <c r="R37" s="4" t="n"/>
+      <c r="S37" s="4" t="inlineStr"/>
+      <c r="T37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2884,6 +3025,8 @@
       <c r="P38" s="4" t="n"/>
       <c r="Q38" s="4" t="n"/>
       <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="inlineStr"/>
+      <c r="T38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2948,6 +3091,8 @@
       </c>
       <c r="Q39" s="4" t="n"/>
       <c r="R39" s="4" t="n"/>
+      <c r="S39" s="4" t="inlineStr"/>
+      <c r="T39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2998,6 +3143,8 @@
       <c r="P40" s="4" t="n"/>
       <c r="Q40" s="4" t="n"/>
       <c r="R40" s="4" t="n"/>
+      <c r="S40" s="4" t="inlineStr"/>
+      <c r="T40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3062,6 +3209,8 @@
       </c>
       <c r="Q41" s="4" t="n"/>
       <c r="R41" s="4" t="n"/>
+      <c r="S41" s="4" t="inlineStr"/>
+      <c r="T41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3112,6 +3261,8 @@
       <c r="P42" s="4" t="n"/>
       <c r="Q42" s="4" t="n"/>
       <c r="R42" s="4" t="n"/>
+      <c r="S42" s="4" t="inlineStr"/>
+      <c r="T42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3176,6 +3327,8 @@
       </c>
       <c r="Q43" s="4" t="n"/>
       <c r="R43" s="4" t="n"/>
+      <c r="S43" s="4" t="inlineStr"/>
+      <c r="T43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3226,6 +3379,8 @@
       <c r="P44" s="4" t="n"/>
       <c r="Q44" s="4" t="n"/>
       <c r="R44" s="4" t="n"/>
+      <c r="S44" s="4" t="inlineStr"/>
+      <c r="T44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3290,6 +3445,8 @@
       </c>
       <c r="Q45" s="4" t="n"/>
       <c r="R45" s="4" t="n"/>
+      <c r="S45" s="4" t="inlineStr"/>
+      <c r="T45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3340,6 +3497,8 @@
       <c r="P46" s="4" t="n"/>
       <c r="Q46" s="4" t="n"/>
       <c r="R46" s="4" t="n"/>
+      <c r="S46" s="4" t="inlineStr"/>
+      <c r="T46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3404,6 +3563,8 @@
       </c>
       <c r="Q47" s="4" t="n"/>
       <c r="R47" s="4" t="n"/>
+      <c r="S47" s="4" t="inlineStr"/>
+      <c r="T47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3454,6 +3615,8 @@
       <c r="P48" s="4" t="n"/>
       <c r="Q48" s="4" t="n"/>
       <c r="R48" s="4" t="n"/>
+      <c r="S48" s="4" t="inlineStr"/>
+      <c r="T48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3497,6 +3660,8 @@
       <c r="P49" s="4" t="n"/>
       <c r="Q49" s="4" t="n"/>
       <c r="R49" s="4" t="n"/>
+      <c r="S49" s="4" t="inlineStr"/>
+      <c r="T49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3561,6 +3726,8 @@
       </c>
       <c r="Q50" s="4" t="n"/>
       <c r="R50" s="4" t="n"/>
+      <c r="S50" s="4" t="inlineStr"/>
+      <c r="T50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3611,6 +3778,8 @@
       <c r="P51" s="4" t="n"/>
       <c r="Q51" s="4" t="n"/>
       <c r="R51" s="4" t="n"/>
+      <c r="S51" s="4" t="inlineStr"/>
+      <c r="T51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3654,6 +3823,8 @@
       <c r="P52" s="4" t="n"/>
       <c r="Q52" s="4" t="n"/>
       <c r="R52" s="4" t="n"/>
+      <c r="S52" s="4" t="inlineStr"/>
+      <c r="T52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3704,6 +3875,8 @@
       <c r="P53" s="4" t="n"/>
       <c r="Q53" s="4" t="n"/>
       <c r="R53" s="4" t="n"/>
+      <c r="S53" s="4" t="inlineStr"/>
+      <c r="T53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3754,6 +3927,8 @@
       <c r="P54" s="4" t="n"/>
       <c r="Q54" s="4" t="n"/>
       <c r="R54" s="4" t="n"/>
+      <c r="S54" s="4" t="inlineStr"/>
+      <c r="T54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3804,6 +3979,8 @@
       <c r="P55" s="4" t="n"/>
       <c r="Q55" s="4" t="n"/>
       <c r="R55" s="4" t="n"/>
+      <c r="S55" s="4" t="inlineStr"/>
+      <c r="T55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3868,6 +4045,8 @@
       </c>
       <c r="Q56" s="4" t="n"/>
       <c r="R56" s="4" t="n"/>
+      <c r="S56" s="4" t="inlineStr"/>
+      <c r="T56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3925,6 +4104,8 @@
       <c r="P57" s="4" t="n"/>
       <c r="Q57" s="4" t="n"/>
       <c r="R57" s="4" t="n"/>
+      <c r="S57" s="4" t="inlineStr"/>
+      <c r="T57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -3975,6 +4156,8 @@
       <c r="P58" s="4" t="n"/>
       <c r="Q58" s="4" t="n"/>
       <c r="R58" s="4" t="n"/>
+      <c r="S58" s="4" t="inlineStr"/>
+      <c r="T58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4025,6 +4208,8 @@
       <c r="P59" s="4" t="n"/>
       <c r="Q59" s="4" t="n"/>
       <c r="R59" s="4" t="n"/>
+      <c r="S59" s="4" t="inlineStr"/>
+      <c r="T59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -4075,6 +4260,8 @@
       <c r="P60" s="4" t="n"/>
       <c r="Q60" s="4" t="n"/>
       <c r="R60" s="4" t="n"/>
+      <c r="S60" s="4" t="inlineStr"/>
+      <c r="T60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4125,6 +4312,8 @@
       <c r="P61" s="4" t="n"/>
       <c r="Q61" s="4" t="n"/>
       <c r="R61" s="4" t="n"/>
+      <c r="S61" s="4" t="inlineStr"/>
+      <c r="T61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4175,6 +4364,8 @@
       <c r="P62" s="4" t="n"/>
       <c r="Q62" s="4" t="n"/>
       <c r="R62" s="4" t="n"/>
+      <c r="S62" s="4" t="inlineStr"/>
+      <c r="T62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4225,6 +4416,8 @@
       <c r="P63" s="4" t="n"/>
       <c r="Q63" s="4" t="n"/>
       <c r="R63" s="4" t="n"/>
+      <c r="S63" s="4" t="inlineStr"/>
+      <c r="T63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -4275,6 +4468,8 @@
       <c r="P64" s="4" t="n"/>
       <c r="Q64" s="4" t="n"/>
       <c r="R64" s="4" t="n"/>
+      <c r="S64" s="4" t="inlineStr"/>
+      <c r="T64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4339,6 +4534,8 @@
       </c>
       <c r="Q65" s="4" t="n"/>
       <c r="R65" s="4" t="n"/>
+      <c r="S65" s="4" t="inlineStr"/>
+      <c r="T65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4403,6 +4600,8 @@
       </c>
       <c r="Q66" s="4" t="n"/>
       <c r="R66" s="4" t="n"/>
+      <c r="S66" s="4" t="inlineStr"/>
+      <c r="T66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -4467,6 +4666,8 @@
       </c>
       <c r="Q67" s="4" t="n"/>
       <c r="R67" s="4" t="n"/>
+      <c r="S67" s="4" t="inlineStr"/>
+      <c r="T67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -4531,6 +4732,8 @@
       </c>
       <c r="Q68" s="4" t="n"/>
       <c r="R68" s="4" t="n"/>
+      <c r="S68" s="4" t="inlineStr"/>
+      <c r="T68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -4581,6 +4784,8 @@
       <c r="P69" s="4" t="n"/>
       <c r="Q69" s="4" t="n"/>
       <c r="R69" s="4" t="n"/>
+      <c r="S69" s="4" t="inlineStr"/>
+      <c r="T69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4645,6 +4850,8 @@
       </c>
       <c r="Q70" s="4" t="n"/>
       <c r="R70" s="4" t="n"/>
+      <c r="S70" s="4" t="inlineStr"/>
+      <c r="T70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4709,6 +4916,8 @@
       </c>
       <c r="Q71" s="4" t="n"/>
       <c r="R71" s="4" t="n"/>
+      <c r="S71" s="4" t="inlineStr"/>
+      <c r="T71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -4759,6 +4968,8 @@
       <c r="P72" s="4" t="n"/>
       <c r="Q72" s="4" t="n"/>
       <c r="R72" s="4" t="n"/>
+      <c r="S72" s="4" t="inlineStr"/>
+      <c r="T72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -4823,6 +5034,8 @@
       </c>
       <c r="Q73" s="4" t="n"/>
       <c r="R73" s="4" t="n"/>
+      <c r="S73" s="4" t="inlineStr"/>
+      <c r="T73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4887,6 +5100,8 @@
       </c>
       <c r="Q74" s="4" t="n"/>
       <c r="R74" s="4" t="n"/>
+      <c r="S74" s="4" t="inlineStr"/>
+      <c r="T74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -4937,6 +5152,8 @@
       <c r="P75" s="4" t="n"/>
       <c r="Q75" s="4" t="n"/>
       <c r="R75" s="4" t="n"/>
+      <c r="S75" s="4" t="inlineStr"/>
+      <c r="T75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -5001,6 +5218,8 @@
       </c>
       <c r="Q76" s="4" t="n"/>
       <c r="R76" s="4" t="n"/>
+      <c r="S76" s="4" t="inlineStr"/>
+      <c r="T76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -5065,6 +5284,8 @@
       </c>
       <c r="Q77" s="4" t="n"/>
       <c r="R77" s="4" t="n"/>
+      <c r="S77" s="4" t="inlineStr"/>
+      <c r="T77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -5115,6 +5336,8 @@
       <c r="P78" s="4" t="n"/>
       <c r="Q78" s="4" t="n"/>
       <c r="R78" s="4" t="n"/>
+      <c r="S78" s="4" t="inlineStr"/>
+      <c r="T78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -5179,6 +5402,8 @@
       </c>
       <c r="Q79" s="4" t="n"/>
       <c r="R79" s="4" t="n"/>
+      <c r="S79" s="4" t="inlineStr"/>
+      <c r="T79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -5243,6 +5468,8 @@
       </c>
       <c r="Q80" s="4" t="n"/>
       <c r="R80" s="4" t="n"/>
+      <c r="S80" s="4" t="inlineStr"/>
+      <c r="T80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -5293,6 +5520,8 @@
       <c r="P81" s="4" t="n"/>
       <c r="Q81" s="4" t="n"/>
       <c r="R81" s="4" t="n"/>
+      <c r="S81" s="4" t="inlineStr"/>
+      <c r="T81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -5357,6 +5586,8 @@
       </c>
       <c r="Q82" s="4" t="n"/>
       <c r="R82" s="4" t="n"/>
+      <c r="S82" s="4" t="inlineStr"/>
+      <c r="T82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -5421,6 +5652,8 @@
       </c>
       <c r="Q83" s="4" t="n"/>
       <c r="R83" s="4" t="n"/>
+      <c r="S83" s="4" t="inlineStr"/>
+      <c r="T83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -5471,6 +5704,8 @@
       <c r="P84" s="4" t="n"/>
       <c r="Q84" s="4" t="n"/>
       <c r="R84" s="4" t="n"/>
+      <c r="S84" s="4" t="inlineStr"/>
+      <c r="T84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -5535,6 +5770,8 @@
       </c>
       <c r="Q85" s="4" t="n"/>
       <c r="R85" s="4" t="n"/>
+      <c r="S85" s="4" t="inlineStr"/>
+      <c r="T85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -5585,6 +5822,8 @@
       <c r="P86" s="4" t="n"/>
       <c r="Q86" s="4" t="n"/>
       <c r="R86" s="4" t="n"/>
+      <c r="S86" s="4" t="inlineStr"/>
+      <c r="T86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -5635,6 +5874,8 @@
       <c r="P87" s="4" t="n"/>
       <c r="Q87" s="4" t="n"/>
       <c r="R87" s="4" t="n"/>
+      <c r="S87" s="4" t="inlineStr"/>
+      <c r="T87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -5685,6 +5926,8 @@
       <c r="P88" s="4" t="n"/>
       <c r="Q88" s="4" t="n"/>
       <c r="R88" s="4" t="n"/>
+      <c r="S88" s="4" t="inlineStr"/>
+      <c r="T88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -5735,6 +5978,8 @@
       <c r="P89" s="4" t="n"/>
       <c r="Q89" s="4" t="n"/>
       <c r="R89" s="4" t="n"/>
+      <c r="S89" s="4" t="inlineStr"/>
+      <c r="T89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -5785,6 +6030,8 @@
       <c r="P90" s="4" t="n"/>
       <c r="Q90" s="4" t="n"/>
       <c r="R90" s="4" t="n"/>
+      <c r="S90" s="4" t="inlineStr"/>
+      <c r="T90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -5835,6 +6082,8 @@
       <c r="P91" s="4" t="n"/>
       <c r="Q91" s="4" t="n"/>
       <c r="R91" s="4" t="n"/>
+      <c r="S91" s="4" t="inlineStr"/>
+      <c r="T91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -5885,6 +6134,8 @@
       <c r="P92" s="4" t="n"/>
       <c r="Q92" s="4" t="n"/>
       <c r="R92" s="4" t="n"/>
+      <c r="S92" s="4" t="inlineStr"/>
+      <c r="T92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -5935,6 +6186,8 @@
       <c r="P93" s="4" t="n"/>
       <c r="Q93" s="4" t="n"/>
       <c r="R93" s="4" t="n"/>
+      <c r="S93" s="4" t="inlineStr"/>
+      <c r="T93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -5999,6 +6252,8 @@
       </c>
       <c r="Q94" s="4" t="n"/>
       <c r="R94" s="4" t="n"/>
+      <c r="S94" s="4" t="inlineStr"/>
+      <c r="T94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -6063,6 +6318,8 @@
       </c>
       <c r="Q95" s="4" t="n"/>
       <c r="R95" s="4" t="n"/>
+      <c r="S95" s="4" t="inlineStr"/>
+      <c r="T95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -6127,6 +6384,8 @@
       </c>
       <c r="Q96" s="4" t="n"/>
       <c r="R96" s="4" t="n"/>
+      <c r="S96" s="4" t="inlineStr"/>
+      <c r="T96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -6191,6 +6450,8 @@
       </c>
       <c r="Q97" s="4" t="n"/>
       <c r="R97" s="4" t="n"/>
+      <c r="S97" s="4" t="inlineStr"/>
+      <c r="T97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -6255,6 +6516,8 @@
       </c>
       <c r="Q98" s="4" t="n"/>
       <c r="R98" s="4" t="n"/>
+      <c r="S98" s="4" t="inlineStr"/>
+      <c r="T98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -6319,6 +6582,8 @@
       </c>
       <c r="Q99" s="4" t="n"/>
       <c r="R99" s="4" t="n"/>
+      <c r="S99" s="4" t="inlineStr"/>
+      <c r="T99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -6383,6 +6648,8 @@
       </c>
       <c r="Q100" s="4" t="n"/>
       <c r="R100" s="4" t="n"/>
+      <c r="S100" s="4" t="inlineStr"/>
+      <c r="T100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -6447,6 +6714,8 @@
       </c>
       <c r="Q101" s="4" t="n"/>
       <c r="R101" s="4" t="n"/>
+      <c r="S101" s="4" t="inlineStr"/>
+      <c r="T101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -6497,6 +6766,8 @@
       <c r="P102" s="4" t="n"/>
       <c r="Q102" s="4" t="n"/>
       <c r="R102" s="4" t="n"/>
+      <c r="S102" s="4" t="inlineStr"/>
+      <c r="T102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -6547,6 +6818,8 @@
       <c r="P103" s="4" t="n"/>
       <c r="Q103" s="4" t="n"/>
       <c r="R103" s="4" t="n"/>
+      <c r="S103" s="4" t="inlineStr"/>
+      <c r="T103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -6597,6 +6870,8 @@
       <c r="P104" s="4" t="n"/>
       <c r="Q104" s="4" t="n"/>
       <c r="R104" s="4" t="n"/>
+      <c r="S104" s="4" t="inlineStr"/>
+      <c r="T104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -6647,6 +6922,8 @@
       <c r="P105" s="4" t="n"/>
       <c r="Q105" s="4" t="n"/>
       <c r="R105" s="4" t="n"/>
+      <c r="S105" s="4" t="inlineStr"/>
+      <c r="T105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -6697,6 +6974,8 @@
       <c r="P106" s="4" t="n"/>
       <c r="Q106" s="4" t="n"/>
       <c r="R106" s="4" t="n"/>
+      <c r="S106" s="4" t="inlineStr"/>
+      <c r="T106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -6761,6 +7040,8 @@
       </c>
       <c r="Q107" s="4" t="n"/>
       <c r="R107" s="4" t="n"/>
+      <c r="S107" s="4" t="inlineStr"/>
+      <c r="T107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -6825,6 +7106,8 @@
       </c>
       <c r="Q108" s="4" t="n"/>
       <c r="R108" s="4" t="n"/>
+      <c r="S108" s="4" t="inlineStr"/>
+      <c r="T108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -6889,6 +7172,8 @@
       </c>
       <c r="Q109" s="4" t="n"/>
       <c r="R109" s="4" t="n"/>
+      <c r="S109" s="4" t="inlineStr"/>
+      <c r="T109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -6953,6 +7238,8 @@
       </c>
       <c r="Q110" s="4" t="n"/>
       <c r="R110" s="4" t="n"/>
+      <c r="S110" s="4" t="inlineStr"/>
+      <c r="T110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -7003,6 +7290,8 @@
       <c r="P111" s="4" t="n"/>
       <c r="Q111" s="4" t="n"/>
       <c r="R111" s="4" t="n"/>
+      <c r="S111" s="4" t="inlineStr"/>
+      <c r="T111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -7053,6 +7342,8 @@
       <c r="P112" s="4" t="n"/>
       <c r="Q112" s="4" t="n"/>
       <c r="R112" s="4" t="n"/>
+      <c r="S112" s="4" t="inlineStr"/>
+      <c r="T112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -7117,6 +7408,8 @@
       </c>
       <c r="Q113" s="4" t="n"/>
       <c r="R113" s="4" t="n"/>
+      <c r="S113" s="4" t="inlineStr"/>
+      <c r="T113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -7181,6 +7474,8 @@
       </c>
       <c r="Q114" s="4" t="n"/>
       <c r="R114" s="4" t="n"/>
+      <c r="S114" s="4" t="inlineStr"/>
+      <c r="T114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -7245,6 +7540,8 @@
       </c>
       <c r="Q115" s="4" t="n"/>
       <c r="R115" s="4" t="n"/>
+      <c r="S115" s="4" t="inlineStr"/>
+      <c r="T115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -7309,6 +7606,8 @@
       </c>
       <c r="Q116" s="4" t="n"/>
       <c r="R116" s="4" t="n"/>
+      <c r="S116" s="4" t="inlineStr"/>
+      <c r="T116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -7359,6 +7658,8 @@
       <c r="P117" s="4" t="n"/>
       <c r="Q117" s="4" t="n"/>
       <c r="R117" s="4" t="n"/>
+      <c r="S117" s="4" t="inlineStr"/>
+      <c r="T117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -7409,6 +7710,8 @@
       <c r="P118" s="4" t="n"/>
       <c r="Q118" s="4" t="n"/>
       <c r="R118" s="4" t="n"/>
+      <c r="S118" s="4" t="inlineStr"/>
+      <c r="T118" s="4" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -7473,6 +7776,8 @@
       </c>
       <c r="Q119" s="4" t="n"/>
       <c r="R119" s="4" t="n"/>
+      <c r="S119" s="4" t="inlineStr"/>
+      <c r="T119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -7537,6 +7842,8 @@
       </c>
       <c r="Q120" s="4" t="n"/>
       <c r="R120" s="4" t="n"/>
+      <c r="S120" s="4" t="inlineStr"/>
+      <c r="T120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -7601,6 +7908,8 @@
       </c>
       <c r="Q121" s="4" t="n"/>
       <c r="R121" s="4" t="n"/>
+      <c r="S121" s="4" t="inlineStr"/>
+      <c r="T121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -7665,6 +7974,8 @@
       </c>
       <c r="Q122" s="4" t="n"/>
       <c r="R122" s="4" t="n"/>
+      <c r="S122" s="4" t="inlineStr"/>
+      <c r="T122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -7715,6 +8026,8 @@
       <c r="P123" s="4" t="n"/>
       <c r="Q123" s="4" t="n"/>
       <c r="R123" s="4" t="n"/>
+      <c r="S123" s="4" t="inlineStr"/>
+      <c r="T123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -7765,6 +8078,8 @@
       <c r="P124" s="4" t="n"/>
       <c r="Q124" s="4" t="n"/>
       <c r="R124" s="4" t="n"/>
+      <c r="S124" s="4" t="inlineStr"/>
+      <c r="T124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -7829,6 +8144,8 @@
       </c>
       <c r="Q125" s="4" t="n"/>
       <c r="R125" s="4" t="n"/>
+      <c r="S125" s="4" t="inlineStr"/>
+      <c r="T125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -7893,6 +8210,8 @@
       </c>
       <c r="Q126" s="4" t="n"/>
       <c r="R126" s="4" t="n"/>
+      <c r="S126" s="4" t="inlineStr"/>
+      <c r="T126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -7957,6 +8276,8 @@
       </c>
       <c r="Q127" s="4" t="n"/>
       <c r="R127" s="4" t="n"/>
+      <c r="S127" s="4" t="inlineStr"/>
+      <c r="T127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -8021,6 +8342,8 @@
       </c>
       <c r="Q128" s="4" t="n"/>
       <c r="R128" s="4" t="n"/>
+      <c r="S128" s="4" t="inlineStr"/>
+      <c r="T128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -8071,6 +8394,8 @@
       <c r="P129" s="4" t="n"/>
       <c r="Q129" s="4" t="n"/>
       <c r="R129" s="4" t="n"/>
+      <c r="S129" s="4" t="inlineStr"/>
+      <c r="T129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -8121,6 +8446,8 @@
       <c r="P130" s="4" t="n"/>
       <c r="Q130" s="4" t="n"/>
       <c r="R130" s="4" t="n"/>
+      <c r="S130" s="4" t="inlineStr"/>
+      <c r="T130" s="4" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -8185,6 +8512,8 @@
       </c>
       <c r="Q131" s="4" t="n"/>
       <c r="R131" s="4" t="n"/>
+      <c r="S131" s="4" t="inlineStr"/>
+      <c r="T131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -8249,6 +8578,8 @@
       </c>
       <c r="Q132" s="4" t="n"/>
       <c r="R132" s="4" t="n"/>
+      <c r="S132" s="4" t="inlineStr"/>
+      <c r="T132" s="4" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -8313,6 +8644,8 @@
       </c>
       <c r="Q133" s="4" t="n"/>
       <c r="R133" s="4" t="n"/>
+      <c r="S133" s="4" t="inlineStr"/>
+      <c r="T133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -8377,6 +8710,8 @@
       </c>
       <c r="Q134" s="4" t="n"/>
       <c r="R134" s="4" t="n"/>
+      <c r="S134" s="4" t="inlineStr"/>
+      <c r="T134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -8427,6 +8762,8 @@
       <c r="P135" s="4" t="n"/>
       <c r="Q135" s="4" t="n"/>
       <c r="R135" s="4" t="n"/>
+      <c r="S135" s="4" t="inlineStr"/>
+      <c r="T135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -8477,6 +8814,8 @@
       <c r="P136" s="4" t="n"/>
       <c r="Q136" s="4" t="n"/>
       <c r="R136" s="4" t="n"/>
+      <c r="S136" s="4" t="inlineStr"/>
+      <c r="T136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -8541,6 +8880,8 @@
       </c>
       <c r="Q137" s="4" t="n"/>
       <c r="R137" s="4" t="n"/>
+      <c r="S137" s="4" t="inlineStr"/>
+      <c r="T137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -8605,6 +8946,8 @@
       </c>
       <c r="Q138" s="4" t="n"/>
       <c r="R138" s="4" t="n"/>
+      <c r="S138" s="4" t="inlineStr"/>
+      <c r="T138" s="4" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -8669,6 +9012,8 @@
       </c>
       <c r="Q139" s="4" t="n"/>
       <c r="R139" s="4" t="n"/>
+      <c r="S139" s="4" t="inlineStr"/>
+      <c r="T139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -8733,6 +9078,8 @@
       </c>
       <c r="Q140" s="4" t="n"/>
       <c r="R140" s="4" t="n"/>
+      <c r="S140" s="4" t="inlineStr"/>
+      <c r="T140" s="4" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -8783,6 +9130,8 @@
       <c r="P141" s="4" t="n"/>
       <c r="Q141" s="4" t="n"/>
       <c r="R141" s="4" t="n"/>
+      <c r="S141" s="4" t="inlineStr"/>
+      <c r="T141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -8833,6 +9182,8 @@
       <c r="P142" s="4" t="n"/>
       <c r="Q142" s="4" t="n"/>
       <c r="R142" s="4" t="n"/>
+      <c r="S142" s="4" t="inlineStr"/>
+      <c r="T142" s="4" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -8897,6 +9248,8 @@
       </c>
       <c r="Q143" s="4" t="n"/>
       <c r="R143" s="4" t="n"/>
+      <c r="S143" s="4" t="inlineStr"/>
+      <c r="T143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -8961,6 +9314,8 @@
       </c>
       <c r="Q144" s="4" t="n"/>
       <c r="R144" s="4" t="n"/>
+      <c r="S144" s="4" t="inlineStr"/>
+      <c r="T144" s="4" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -9025,6 +9380,8 @@
       </c>
       <c r="Q145" s="4" t="n"/>
       <c r="R145" s="4" t="n"/>
+      <c r="S145" s="4" t="inlineStr"/>
+      <c r="T145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -9089,6 +9446,8 @@
       </c>
       <c r="Q146" s="4" t="n"/>
       <c r="R146" s="4" t="n"/>
+      <c r="S146" s="4" t="inlineStr"/>
+      <c r="T146" s="4" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -9139,6 +9498,8 @@
       <c r="P147" s="4" t="n"/>
       <c r="Q147" s="4" t="n"/>
       <c r="R147" s="4" t="n"/>
+      <c r="S147" s="4" t="inlineStr"/>
+      <c r="T147" s="4" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -9189,6 +9550,8 @@
       <c r="P148" s="4" t="n"/>
       <c r="Q148" s="4" t="n"/>
       <c r="R148" s="4" t="n"/>
+      <c r="S148" s="4" t="inlineStr"/>
+      <c r="T148" s="4" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -9253,6 +9616,8 @@
       </c>
       <c r="Q149" s="4" t="n"/>
       <c r="R149" s="4" t="n"/>
+      <c r="S149" s="4" t="inlineStr"/>
+      <c r="T149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -9317,6 +9682,8 @@
       </c>
       <c r="Q150" s="4" t="n"/>
       <c r="R150" s="4" t="n"/>
+      <c r="S150" s="4" t="inlineStr"/>
+      <c r="T150" s="4" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -9381,6 +9748,8 @@
       </c>
       <c r="Q151" s="4" t="n"/>
       <c r="R151" s="4" t="n"/>
+      <c r="S151" s="4" t="inlineStr"/>
+      <c r="T151" s="4" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -9445,6 +9814,8 @@
       </c>
       <c r="Q152" s="4" t="n"/>
       <c r="R152" s="4" t="n"/>
+      <c r="S152" s="4" t="inlineStr"/>
+      <c r="T152" s="4" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -9495,6 +9866,8 @@
       <c r="P153" s="4" t="n"/>
       <c r="Q153" s="4" t="n"/>
       <c r="R153" s="4" t="n"/>
+      <c r="S153" s="4" t="inlineStr"/>
+      <c r="T153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -9545,6 +9918,8 @@
       <c r="P154" s="4" t="n"/>
       <c r="Q154" s="4" t="n"/>
       <c r="R154" s="4" t="n"/>
+      <c r="S154" s="4" t="inlineStr"/>
+      <c r="T154" s="4" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -9609,6 +9984,8 @@
       </c>
       <c r="Q155" s="4" t="n"/>
       <c r="R155" s="4" t="n"/>
+      <c r="S155" s="4" t="inlineStr"/>
+      <c r="T155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -9673,6 +10050,8 @@
       </c>
       <c r="Q156" s="4" t="n"/>
       <c r="R156" s="4" t="n"/>
+      <c r="S156" s="4" t="inlineStr"/>
+      <c r="T156" s="4" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -9737,6 +10116,8 @@
       </c>
       <c r="Q157" s="4" t="n"/>
       <c r="R157" s="4" t="n"/>
+      <c r="S157" s="4" t="inlineStr"/>
+      <c r="T157" s="4" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -9801,6 +10182,8 @@
       </c>
       <c r="Q158" s="4" t="n"/>
       <c r="R158" s="4" t="n"/>
+      <c r="S158" s="4" t="inlineStr"/>
+      <c r="T158" s="4" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -9851,6 +10234,8 @@
       <c r="P159" s="4" t="n"/>
       <c r="Q159" s="4" t="n"/>
       <c r="R159" s="4" t="n"/>
+      <c r="S159" s="4" t="inlineStr"/>
+      <c r="T159" s="4" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -9901,6 +10286,8 @@
       <c r="P160" s="4" t="n"/>
       <c r="Q160" s="4" t="n"/>
       <c r="R160" s="4" t="n"/>
+      <c r="S160" s="4" t="inlineStr"/>
+      <c r="T160" s="4" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -9965,6 +10352,8 @@
       </c>
       <c r="Q161" s="4" t="n"/>
       <c r="R161" s="4" t="n"/>
+      <c r="S161" s="4" t="inlineStr"/>
+      <c r="T161" s="4" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -10029,6 +10418,8 @@
       </c>
       <c r="Q162" s="4" t="n"/>
       <c r="R162" s="4" t="n"/>
+      <c r="S162" s="4" t="inlineStr"/>
+      <c r="T162" s="4" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -10093,6 +10484,8 @@
       </c>
       <c r="Q163" s="4" t="n"/>
       <c r="R163" s="4" t="n"/>
+      <c r="S163" s="4" t="inlineStr"/>
+      <c r="T163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -10157,6 +10550,8 @@
       </c>
       <c r="Q164" s="4" t="n"/>
       <c r="R164" s="4" t="n"/>
+      <c r="S164" s="4" t="inlineStr"/>
+      <c r="T164" s="4" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -10207,6 +10602,8 @@
       <c r="P165" s="4" t="n"/>
       <c r="Q165" s="4" t="n"/>
       <c r="R165" s="4" t="n"/>
+      <c r="S165" s="4" t="inlineStr"/>
+      <c r="T165" s="4" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -10257,6 +10654,8 @@
       <c r="P166" s="4" t="n"/>
       <c r="Q166" s="4" t="n"/>
       <c r="R166" s="4" t="n"/>
+      <c r="S166" s="4" t="inlineStr"/>
+      <c r="T166" s="4" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -10321,6 +10720,8 @@
       </c>
       <c r="Q167" s="4" t="n"/>
       <c r="R167" s="4" t="n"/>
+      <c r="S167" s="4" t="inlineStr"/>
+      <c r="T167" s="4" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -10371,6 +10772,8 @@
       <c r="P168" s="4" t="n"/>
       <c r="Q168" s="4" t="n"/>
       <c r="R168" s="4" t="n"/>
+      <c r="S168" s="4" t="inlineStr"/>
+      <c r="T168" s="4" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -10421,6 +10824,8 @@
       <c r="P169" s="4" t="n"/>
       <c r="Q169" s="4" t="n"/>
       <c r="R169" s="4" t="n"/>
+      <c r="S169" s="4" t="inlineStr"/>
+      <c r="T169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -10471,6 +10876,8 @@
       <c r="P170" s="4" t="n"/>
       <c r="Q170" s="4" t="n"/>
       <c r="R170" s="4" t="n"/>
+      <c r="S170" s="4" t="inlineStr"/>
+      <c r="T170" s="4" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -10521,6 +10928,8 @@
       <c r="P171" s="4" t="n"/>
       <c r="Q171" s="4" t="n"/>
       <c r="R171" s="4" t="n"/>
+      <c r="S171" s="4" t="inlineStr"/>
+      <c r="T171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -10571,6 +10980,8 @@
       <c r="P172" s="4" t="n"/>
       <c r="Q172" s="4" t="n"/>
       <c r="R172" s="4" t="n"/>
+      <c r="S172" s="4" t="inlineStr"/>
+      <c r="T172" s="4" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -10635,6 +11046,8 @@
       </c>
       <c r="Q173" s="4" t="n"/>
       <c r="R173" s="4" t="n"/>
+      <c r="S173" s="4" t="inlineStr"/>
+      <c r="T173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -10678,6 +11091,8 @@
       <c r="P174" s="4" t="n"/>
       <c r="Q174" s="4" t="n"/>
       <c r="R174" s="4" t="n"/>
+      <c r="S174" s="4" t="inlineStr"/>
+      <c r="T174" s="4" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -10742,6 +11157,8 @@
       </c>
       <c r="Q175" s="4" t="n"/>
       <c r="R175" s="4" t="n"/>
+      <c r="S175" s="4" t="inlineStr"/>
+      <c r="T175" s="4" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -10806,6 +11223,8 @@
       </c>
       <c r="Q176" s="4" t="n"/>
       <c r="R176" s="4" t="n"/>
+      <c r="S176" s="4" t="inlineStr"/>
+      <c r="T176" s="4" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -10849,6 +11268,8 @@
       <c r="P177" s="4" t="n"/>
       <c r="Q177" s="4" t="n"/>
       <c r="R177" s="4" t="n"/>
+      <c r="S177" s="4" t="inlineStr"/>
+      <c r="T177" s="4" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -10913,6 +11334,8 @@
       </c>
       <c r="Q178" s="4" t="n"/>
       <c r="R178" s="4" t="n"/>
+      <c r="S178" s="4" t="inlineStr"/>
+      <c r="T178" s="4" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -10977,6 +11400,8 @@
       </c>
       <c r="Q179" s="4" t="n"/>
       <c r="R179" s="4" t="n"/>
+      <c r="S179" s="4" t="inlineStr"/>
+      <c r="T179" s="4" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -11020,6 +11445,8 @@
       <c r="P180" s="4" t="n"/>
       <c r="Q180" s="4" t="n"/>
       <c r="R180" s="4" t="n"/>
+      <c r="S180" s="4" t="inlineStr"/>
+      <c r="T180" s="4" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -11084,6 +11511,8 @@
       </c>
       <c r="Q181" s="4" t="n"/>
       <c r="R181" s="4" t="n"/>
+      <c r="S181" s="4" t="inlineStr"/>
+      <c r="T181" s="4" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -11134,6 +11563,8 @@
       <c r="P182" s="4" t="n"/>
       <c r="Q182" s="4" t="n"/>
       <c r="R182" s="4" t="n"/>
+      <c r="S182" s="4" t="inlineStr"/>
+      <c r="T182" s="4" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -11184,6 +11615,8 @@
       <c r="P183" s="4" t="n"/>
       <c r="Q183" s="4" t="n"/>
       <c r="R183" s="4" t="n"/>
+      <c r="S183" s="4" t="inlineStr"/>
+      <c r="T183" s="4" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -11234,6 +11667,8 @@
       <c r="P184" s="4" t="n"/>
       <c r="Q184" s="4" t="n"/>
       <c r="R184" s="4" t="n"/>
+      <c r="S184" s="4" t="inlineStr"/>
+      <c r="T184" s="4" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -11284,6 +11719,8 @@
       <c r="P185" s="4" t="n"/>
       <c r="Q185" s="4" t="n"/>
       <c r="R185" s="4" t="n"/>
+      <c r="S185" s="4" t="inlineStr"/>
+      <c r="T185" s="4" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -11348,6 +11785,8 @@
       </c>
       <c r="Q186" s="4" t="n"/>
       <c r="R186" s="4" t="n"/>
+      <c r="S186" s="4" t="inlineStr"/>
+      <c r="T186" s="4" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -11412,6 +11851,8 @@
       </c>
       <c r="Q187" s="4" t="n"/>
       <c r="R187" s="4" t="n"/>
+      <c r="S187" s="4" t="inlineStr"/>
+      <c r="T187" s="4" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -11476,6 +11917,8 @@
       </c>
       <c r="Q188" s="4" t="n"/>
       <c r="R188" s="4" t="n"/>
+      <c r="S188" s="4" t="inlineStr"/>
+      <c r="T188" s="4" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -11540,6 +11983,8 @@
       </c>
       <c r="Q189" s="4" t="n"/>
       <c r="R189" s="4" t="n"/>
+      <c r="S189" s="4" t="inlineStr"/>
+      <c r="T189" s="4" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -11604,6 +12049,8 @@
       </c>
       <c r="Q190" s="4" t="n"/>
       <c r="R190" s="4" t="n"/>
+      <c r="S190" s="4" t="inlineStr"/>
+      <c r="T190" s="4" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -11668,6 +12115,8 @@
       </c>
       <c r="Q191" s="4" t="n"/>
       <c r="R191" s="4" t="n"/>
+      <c r="S191" s="4" t="inlineStr"/>
+      <c r="T191" s="4" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -11732,6 +12181,8 @@
       </c>
       <c r="Q192" s="4" t="n"/>
       <c r="R192" s="4" t="n"/>
+      <c r="S192" s="4" t="inlineStr"/>
+      <c r="T192" s="4" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
@@ -11796,6 +12247,8 @@
       </c>
       <c r="Q193" s="4" t="n"/>
       <c r="R193" s="4" t="n"/>
+      <c r="S193" s="4" t="inlineStr"/>
+      <c r="T193" s="4" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
@@ -11846,6 +12299,8 @@
       <c r="P194" s="4" t="n"/>
       <c r="Q194" s="4" t="n"/>
       <c r="R194" s="4" t="n"/>
+      <c r="S194" s="4" t="inlineStr"/>
+      <c r="T194" s="4" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
@@ -11896,6 +12351,8 @@
       <c r="P195" s="4" t="n"/>
       <c r="Q195" s="4" t="n"/>
       <c r="R195" s="4" t="n"/>
+      <c r="S195" s="4" t="inlineStr"/>
+      <c r="T195" s="4" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -11960,6 +12417,8 @@
       </c>
       <c r="Q196" s="4" t="n"/>
       <c r="R196" s="4" t="n"/>
+      <c r="S196" s="4" t="inlineStr"/>
+      <c r="T196" s="4" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -12024,6 +12483,8 @@
       </c>
       <c r="Q197" s="4" t="n"/>
       <c r="R197" s="4" t="n"/>
+      <c r="S197" s="4" t="inlineStr"/>
+      <c r="T197" s="4" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -12088,6 +12549,8 @@
       </c>
       <c r="Q198" s="4" t="n"/>
       <c r="R198" s="4" t="n"/>
+      <c r="S198" s="4" t="inlineStr"/>
+      <c r="T198" s="4" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -12152,6 +12615,8 @@
       </c>
       <c r="Q199" s="4" t="n"/>
       <c r="R199" s="4" t="n"/>
+      <c r="S199" s="4" t="inlineStr"/>
+      <c r="T199" s="4" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -12216,6 +12681,8 @@
       </c>
       <c r="Q200" s="4" t="n"/>
       <c r="R200" s="4" t="n"/>
+      <c r="S200" s="4" t="inlineStr"/>
+      <c r="T200" s="4" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -12280,6 +12747,8 @@
       </c>
       <c r="Q201" s="4" t="n"/>
       <c r="R201" s="4" t="n"/>
+      <c r="S201" s="4" t="inlineStr"/>
+      <c r="T201" s="4" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
@@ -12344,6 +12813,8 @@
       </c>
       <c r="Q202" s="4" t="n"/>
       <c r="R202" s="4" t="n"/>
+      <c r="S202" s="4" t="inlineStr"/>
+      <c r="T202" s="4" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
@@ -12408,6 +12879,8 @@
       </c>
       <c r="Q203" s="4" t="n"/>
       <c r="R203" s="4" t="n"/>
+      <c r="S203" s="4" t="inlineStr"/>
+      <c r="T203" s="4" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
@@ -12472,6 +12945,8 @@
       </c>
       <c r="Q204" s="4" t="n"/>
       <c r="R204" s="4" t="n"/>
+      <c r="S204" s="4" t="inlineStr"/>
+      <c r="T204" s="4" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -12536,6 +13011,8 @@
       </c>
       <c r="Q205" s="4" t="n"/>
       <c r="R205" s="4" t="n"/>
+      <c r="S205" s="4" t="inlineStr"/>
+      <c r="T205" s="4" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
@@ -12600,6 +13077,8 @@
       </c>
       <c r="Q206" s="4" t="n"/>
       <c r="R206" s="4" t="n"/>
+      <c r="S206" s="4" t="inlineStr"/>
+      <c r="T206" s="4" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -12664,6 +13143,8 @@
       </c>
       <c r="Q207" s="4" t="n"/>
       <c r="R207" s="4" t="n"/>
+      <c r="S207" s="4" t="inlineStr"/>
+      <c r="T207" s="4" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
@@ -12728,6 +13209,8 @@
       </c>
       <c r="Q208" s="4" t="n"/>
       <c r="R208" s="4" t="n"/>
+      <c r="S208" s="4" t="inlineStr"/>
+      <c r="T208" s="4" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
@@ -12792,6 +13275,8 @@
       </c>
       <c r="Q209" s="4" t="n"/>
       <c r="R209" s="4" t="n"/>
+      <c r="S209" s="4" t="inlineStr"/>
+      <c r="T209" s="4" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
@@ -12842,6 +13327,8 @@
       <c r="P210" s="4" t="n"/>
       <c r="Q210" s="4" t="n"/>
       <c r="R210" s="4" t="n"/>
+      <c r="S210" s="4" t="inlineStr"/>
+      <c r="T210" s="4" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
@@ -12892,6 +13379,8 @@
       <c r="P211" s="4" t="n"/>
       <c r="Q211" s="4" t="n"/>
       <c r="R211" s="4" t="n"/>
+      <c r="S211" s="4" t="inlineStr"/>
+      <c r="T211" s="4" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
@@ -12956,6 +13445,8 @@
       </c>
       <c r="Q212" s="4" t="n"/>
       <c r="R212" s="4" t="n"/>
+      <c r="S212" s="4" t="inlineStr"/>
+      <c r="T212" s="4" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
@@ -13006,6 +13497,8 @@
       <c r="P213" s="4" t="n"/>
       <c r="Q213" s="4" t="n"/>
       <c r="R213" s="4" t="n"/>
+      <c r="S213" s="4" t="inlineStr"/>
+      <c r="T213" s="4" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
@@ -13056,6 +13549,8 @@
       <c r="P214" s="4" t="n"/>
       <c r="Q214" s="4" t="n"/>
       <c r="R214" s="4" t="n"/>
+      <c r="S214" s="4" t="inlineStr"/>
+      <c r="T214" s="4" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -13106,6 +13601,8 @@
       <c r="P215" s="4" t="n"/>
       <c r="Q215" s="4" t="n"/>
       <c r="R215" s="4" t="n"/>
+      <c r="S215" s="4" t="inlineStr"/>
+      <c r="T215" s="4" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
@@ -13170,6 +13667,8 @@
       </c>
       <c r="Q216" s="4" t="n"/>
       <c r="R216" s="4" t="n"/>
+      <c r="S216" s="4" t="inlineStr"/>
+      <c r="T216" s="4" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
@@ -13220,6 +13719,8 @@
       <c r="P217" s="4" t="n"/>
       <c r="Q217" s="4" t="n"/>
       <c r="R217" s="4" t="n"/>
+      <c r="S217" s="4" t="inlineStr"/>
+      <c r="T217" s="4" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
@@ -13284,6 +13785,8 @@
       </c>
       <c r="Q218" s="4" t="n"/>
       <c r="R218" s="4" t="n"/>
+      <c r="S218" s="4" t="inlineStr"/>
+      <c r="T218" s="4" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
@@ -13334,6 +13837,8 @@
       <c r="P219" s="4" t="n"/>
       <c r="Q219" s="4" t="n"/>
       <c r="R219" s="4" t="n"/>
+      <c r="S219" s="4" t="inlineStr"/>
+      <c r="T219" s="4" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
@@ -13384,6 +13889,8 @@
       <c r="P220" s="4" t="n"/>
       <c r="Q220" s="4" t="n"/>
       <c r="R220" s="4" t="n"/>
+      <c r="S220" s="4" t="inlineStr"/>
+      <c r="T220" s="4" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
@@ -13434,6 +13941,8 @@
       <c r="P221" s="4" t="n"/>
       <c r="Q221" s="4" t="n"/>
       <c r="R221" s="4" t="n"/>
+      <c r="S221" s="4" t="inlineStr"/>
+      <c r="T221" s="4" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
@@ -13484,6 +13993,8 @@
       <c r="P222" s="4" t="n"/>
       <c r="Q222" s="4" t="n"/>
       <c r="R222" s="4" t="n"/>
+      <c r="S222" s="4" t="inlineStr"/>
+      <c r="T222" s="4" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
@@ -13534,6 +14045,8 @@
       <c r="P223" s="4" t="n"/>
       <c r="Q223" s="4" t="n"/>
       <c r="R223" s="4" t="n"/>
+      <c r="S223" s="4" t="inlineStr"/>
+      <c r="T223" s="4" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
@@ -13584,6 +14097,8 @@
       <c r="P224" s="4" t="n"/>
       <c r="Q224" s="4" t="n"/>
       <c r="R224" s="4" t="n"/>
+      <c r="S224" s="4" t="inlineStr"/>
+      <c r="T224" s="4" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
@@ -13634,6 +14149,8 @@
       <c r="P225" s="4" t="n"/>
       <c r="Q225" s="4" t="n"/>
       <c r="R225" s="4" t="n"/>
+      <c r="S225" s="4" t="inlineStr"/>
+      <c r="T225" s="4" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
@@ -13684,6 +14201,8 @@
       <c r="P226" s="4" t="n"/>
       <c r="Q226" s="4" t="n"/>
       <c r="R226" s="4" t="n"/>
+      <c r="S226" s="4" t="inlineStr"/>
+      <c r="T226" s="4" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
@@ -13748,6 +14267,8 @@
       </c>
       <c r="Q227" s="4" t="n"/>
       <c r="R227" s="4" t="n"/>
+      <c r="S227" s="4" t="inlineStr"/>
+      <c r="T227" s="4" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
@@ -13798,6 +14319,8 @@
       <c r="P228" s="4" t="n"/>
       <c r="Q228" s="4" t="n"/>
       <c r="R228" s="4" t="n"/>
+      <c r="S228" s="4" t="inlineStr"/>
+      <c r="T228" s="4" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
@@ -13841,6 +14364,8 @@
       <c r="P229" s="4" t="n"/>
       <c r="Q229" s="4" t="n"/>
       <c r="R229" s="4" t="n"/>
+      <c r="S229" s="4" t="inlineStr"/>
+      <c r="T229" s="4" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
@@ -13905,6 +14430,8 @@
       </c>
       <c r="Q230" s="4" t="n"/>
       <c r="R230" s="4" t="n"/>
+      <c r="S230" s="4" t="inlineStr"/>
+      <c r="T230" s="4" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
@@ -13955,6 +14482,8 @@
       <c r="P231" s="4" t="n"/>
       <c r="Q231" s="4" t="n"/>
       <c r="R231" s="4" t="n"/>
+      <c r="S231" s="4" t="inlineStr"/>
+      <c r="T231" s="4" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
@@ -13998,6 +14527,8 @@
       <c r="P232" s="4" t="n"/>
       <c r="Q232" s="4" t="n"/>
       <c r="R232" s="4" t="n"/>
+      <c r="S232" s="4" t="inlineStr"/>
+      <c r="T232" s="4" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
@@ -14062,6 +14593,8 @@
       </c>
       <c r="Q233" s="4" t="n"/>
       <c r="R233" s="4" t="n"/>
+      <c r="S233" s="4" t="inlineStr"/>
+      <c r="T233" s="4" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
@@ -14112,6 +14645,8 @@
       <c r="P234" s="4" t="n"/>
       <c r="Q234" s="4" t="n"/>
       <c r="R234" s="4" t="n"/>
+      <c r="S234" s="4" t="inlineStr"/>
+      <c r="T234" s="4" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
@@ -14155,6 +14690,8 @@
       <c r="P235" s="4" t="n"/>
       <c r="Q235" s="4" t="n"/>
       <c r="R235" s="4" t="n"/>
+      <c r="S235" s="4" t="inlineStr"/>
+      <c r="T235" s="4" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
@@ -14219,6 +14756,8 @@
       </c>
       <c r="Q236" s="4" t="n"/>
       <c r="R236" s="4" t="n"/>
+      <c r="S236" s="4" t="inlineStr"/>
+      <c r="T236" s="4" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
@@ -14269,6 +14808,8 @@
       <c r="P237" s="4" t="n"/>
       <c r="Q237" s="4" t="n"/>
       <c r="R237" s="4" t="n"/>
+      <c r="S237" s="4" t="inlineStr"/>
+      <c r="T237" s="4" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
@@ -14333,6 +14874,8 @@
       </c>
       <c r="Q238" s="4" t="n"/>
       <c r="R238" s="4" t="n"/>
+      <c r="S238" s="4" t="inlineStr"/>
+      <c r="T238" s="4" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
@@ -14383,6 +14926,8 @@
       <c r="P239" s="4" t="n"/>
       <c r="Q239" s="4" t="n"/>
       <c r="R239" s="4" t="n"/>
+      <c r="S239" s="4" t="inlineStr"/>
+      <c r="T239" s="4" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
@@ -14447,6 +14992,8 @@
       </c>
       <c r="Q240" s="4" t="n"/>
       <c r="R240" s="4" t="n"/>
+      <c r="S240" s="4" t="inlineStr"/>
+      <c r="T240" s="4" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
@@ -14497,6 +15044,8 @@
       <c r="P241" s="4" t="n"/>
       <c r="Q241" s="4" t="n"/>
       <c r="R241" s="4" t="n"/>
+      <c r="S241" s="4" t="inlineStr"/>
+      <c r="T241" s="4" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
@@ -14561,6 +15110,8 @@
       </c>
       <c r="Q242" s="4" t="n"/>
       <c r="R242" s="4" t="n"/>
+      <c r="S242" s="4" t="inlineStr"/>
+      <c r="T242" s="4" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
@@ -14611,6 +15162,8 @@
       <c r="P243" s="4" t="n"/>
       <c r="Q243" s="4" t="n"/>
       <c r="R243" s="4" t="n"/>
+      <c r="S243" s="4" t="inlineStr"/>
+      <c r="T243" s="4" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
@@ -14675,6 +15228,8 @@
       </c>
       <c r="Q244" s="4" t="n"/>
       <c r="R244" s="4" t="n"/>
+      <c r="S244" s="4" t="inlineStr"/>
+      <c r="T244" s="4" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
@@ -14725,6 +15280,8 @@
       <c r="P245" s="4" t="n"/>
       <c r="Q245" s="4" t="n"/>
       <c r="R245" s="4" t="n"/>
+      <c r="S245" s="4" t="inlineStr"/>
+      <c r="T245" s="4" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
@@ -14775,6 +15332,8 @@
       <c r="P246" s="4" t="n"/>
       <c r="Q246" s="4" t="n"/>
       <c r="R246" s="4" t="n"/>
+      <c r="S246" s="4" t="inlineStr"/>
+      <c r="T246" s="4" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
@@ -14832,6 +15391,8 @@
       <c r="P247" s="4" t="n"/>
       <c r="Q247" s="4" t="n"/>
       <c r="R247" s="4" t="n"/>
+      <c r="S247" s="4" t="inlineStr"/>
+      <c r="T247" s="4" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
@@ -14882,6 +15443,8 @@
       <c r="P248" s="4" t="n"/>
       <c r="Q248" s="4" t="n"/>
       <c r="R248" s="4" t="n"/>
+      <c r="S248" s="4" t="inlineStr"/>
+      <c r="T248" s="4" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
@@ -14939,6 +15502,8 @@
       <c r="P249" s="4" t="n"/>
       <c r="Q249" s="4" t="n"/>
       <c r="R249" s="4" t="n"/>
+      <c r="S249" s="4" t="inlineStr"/>
+      <c r="T249" s="4" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
@@ -14989,6 +15554,8 @@
       <c r="P250" s="4" t="n"/>
       <c r="Q250" s="4" t="n"/>
       <c r="R250" s="4" t="n"/>
+      <c r="S250" s="4" t="inlineStr"/>
+      <c r="T250" s="4" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
@@ -15046,6 +15613,8 @@
       <c r="P251" s="4" t="n"/>
       <c r="Q251" s="4" t="n"/>
       <c r="R251" s="4" t="n"/>
+      <c r="S251" s="4" t="inlineStr"/>
+      <c r="T251" s="4" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
@@ -15096,6 +15665,8 @@
       <c r="P252" s="4" t="n"/>
       <c r="Q252" s="4" t="n"/>
       <c r="R252" s="4" t="n"/>
+      <c r="S252" s="4" t="inlineStr"/>
+      <c r="T252" s="4" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
@@ -15153,6 +15724,8 @@
       <c r="P253" s="4" t="n"/>
       <c r="Q253" s="4" t="n"/>
       <c r="R253" s="4" t="n"/>
+      <c r="S253" s="4" t="inlineStr"/>
+      <c r="T253" s="4" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
@@ -15203,6 +15776,8 @@
       <c r="P254" s="4" t="n"/>
       <c r="Q254" s="4" t="n"/>
       <c r="R254" s="4" t="n"/>
+      <c r="S254" s="4" t="inlineStr"/>
+      <c r="T254" s="4" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
@@ -15260,6 +15835,8 @@
       <c r="P255" s="4" t="n"/>
       <c r="Q255" s="4" t="n"/>
       <c r="R255" s="4" t="n"/>
+      <c r="S255" s="4" t="inlineStr"/>
+      <c r="T255" s="4" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
@@ -15310,6 +15887,8 @@
       <c r="P256" s="4" t="n"/>
       <c r="Q256" s="4" t="n"/>
       <c r="R256" s="4" t="n"/>
+      <c r="S256" s="4" t="inlineStr"/>
+      <c r="T256" s="4" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
@@ -15360,6 +15939,8 @@
       <c r="P257" s="4" t="n"/>
       <c r="Q257" s="4" t="n"/>
       <c r="R257" s="4" t="n"/>
+      <c r="S257" s="4" t="inlineStr"/>
+      <c r="T257" s="4" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
@@ -15410,6 +15991,8 @@
       <c r="P258" s="4" t="n"/>
       <c r="Q258" s="4" t="n"/>
       <c r="R258" s="4" t="n"/>
+      <c r="S258" s="4" t="inlineStr"/>
+      <c r="T258" s="4" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
@@ -15474,6 +16057,8 @@
       </c>
       <c r="Q259" s="4" t="n"/>
       <c r="R259" s="4" t="n"/>
+      <c r="S259" s="4" t="inlineStr"/>
+      <c r="T259" s="4" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
@@ -15538,6 +16123,8 @@
       </c>
       <c r="Q260" s="4" t="n"/>
       <c r="R260" s="4" t="n"/>
+      <c r="S260" s="4" t="inlineStr"/>
+      <c r="T260" s="4" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
@@ -15602,6 +16189,8 @@
       </c>
       <c r="Q261" s="4" t="n"/>
       <c r="R261" s="4" t="n"/>
+      <c r="S261" s="4" t="inlineStr"/>
+      <c r="T261" s="4" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
@@ -15666,6 +16255,8 @@
       </c>
       <c r="Q262" s="4" t="n"/>
       <c r="R262" s="4" t="n"/>
+      <c r="S262" s="4" t="inlineStr"/>
+      <c r="T262" s="4" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
@@ -15716,6 +16307,8 @@
       <c r="P263" s="4" t="n"/>
       <c r="Q263" s="4" t="n"/>
       <c r="R263" s="4" t="n"/>
+      <c r="S263" s="4" t="inlineStr"/>
+      <c r="T263" s="4" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
@@ -15766,6 +16359,8 @@
       <c r="P264" s="4" t="n"/>
       <c r="Q264" s="4" t="n"/>
       <c r="R264" s="4" t="n"/>
+      <c r="S264" s="4" t="inlineStr"/>
+      <c r="T264" s="4" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
@@ -15816,6 +16411,8 @@
       <c r="P265" s="4" t="n"/>
       <c r="Q265" s="4" t="n"/>
       <c r="R265" s="4" t="n"/>
+      <c r="S265" s="4" t="inlineStr"/>
+      <c r="T265" s="4" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
@@ -15866,6 +16463,8 @@
       <c r="P266" s="4" t="n"/>
       <c r="Q266" s="4" t="n"/>
       <c r="R266" s="4" t="n"/>
+      <c r="S266" s="4" t="inlineStr"/>
+      <c r="T266" s="4" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
@@ -15916,6 +16515,8 @@
       <c r="P267" s="4" t="n"/>
       <c r="Q267" s="4" t="n"/>
       <c r="R267" s="4" t="n"/>
+      <c r="S267" s="4" t="inlineStr"/>
+      <c r="T267" s="4" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
@@ -15966,6 +16567,8 @@
       <c r="P268" s="4" t="n"/>
       <c r="Q268" s="4" t="n"/>
       <c r="R268" s="4" t="n"/>
+      <c r="S268" s="4" t="inlineStr"/>
+      <c r="T268" s="4" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
@@ -16016,6 +16619,8 @@
       <c r="P269" s="4" t="n"/>
       <c r="Q269" s="4" t="n"/>
       <c r="R269" s="4" t="n"/>
+      <c r="S269" s="4" t="inlineStr"/>
+      <c r="T269" s="4" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
@@ -16066,6 +16671,8 @@
       <c r="P270" s="4" t="n"/>
       <c r="Q270" s="4" t="n"/>
       <c r="R270" s="4" t="n"/>
+      <c r="S270" s="4" t="inlineStr"/>
+      <c r="T270" s="4" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
@@ -16116,6 +16723,8 @@
       <c r="P271" s="4" t="n"/>
       <c r="Q271" s="4" t="n"/>
       <c r="R271" s="4" t="n"/>
+      <c r="S271" s="4" t="inlineStr"/>
+      <c r="T271" s="4" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
@@ -16166,6 +16775,8 @@
       <c r="P272" s="4" t="n"/>
       <c r="Q272" s="4" t="n"/>
       <c r="R272" s="4" t="n"/>
+      <c r="S272" s="4" t="inlineStr"/>
+      <c r="T272" s="4" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
@@ -16230,6 +16841,8 @@
       </c>
       <c r="Q273" s="4" t="n"/>
       <c r="R273" s="4" t="n"/>
+      <c r="S273" s="4" t="inlineStr"/>
+      <c r="T273" s="4" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
@@ -16280,6 +16893,8 @@
       <c r="P274" s="4" t="n"/>
       <c r="Q274" s="4" t="n"/>
       <c r="R274" s="4" t="n"/>
+      <c r="S274" s="4" t="inlineStr"/>
+      <c r="T274" s="4" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
@@ -16344,6 +16959,8 @@
       </c>
       <c r="Q275" s="4" t="n"/>
       <c r="R275" s="4" t="n"/>
+      <c r="S275" s="4" t="inlineStr"/>
+      <c r="T275" s="4" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
@@ -16394,6 +17011,8 @@
       <c r="P276" s="4" t="n"/>
       <c r="Q276" s="4" t="n"/>
       <c r="R276" s="4" t="n"/>
+      <c r="S276" s="4" t="inlineStr"/>
+      <c r="T276" s="4" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
@@ -16458,6 +17077,8 @@
       </c>
       <c r="Q277" s="4" t="n"/>
       <c r="R277" s="4" t="n"/>
+      <c r="S277" s="4" t="inlineStr"/>
+      <c r="T277" s="4" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
@@ -16508,6 +17129,8 @@
       <c r="P278" s="4" t="n"/>
       <c r="Q278" s="4" t="n"/>
       <c r="R278" s="4" t="n"/>
+      <c r="S278" s="4" t="inlineStr"/>
+      <c r="T278" s="4" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
@@ -16572,6 +17195,8 @@
       </c>
       <c r="Q279" s="4" t="n"/>
       <c r="R279" s="4" t="n"/>
+      <c r="S279" s="4" t="inlineStr"/>
+      <c r="T279" s="4" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
@@ -16622,6 +17247,8 @@
       <c r="P280" s="4" t="n"/>
       <c r="Q280" s="4" t="n"/>
       <c r="R280" s="4" t="n"/>
+      <c r="S280" s="4" t="inlineStr"/>
+      <c r="T280" s="4" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
@@ -16686,6 +17313,8 @@
       </c>
       <c r="Q281" s="4" t="n"/>
       <c r="R281" s="4" t="n"/>
+      <c r="S281" s="4" t="inlineStr"/>
+      <c r="T281" s="4" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
@@ -16750,6 +17379,8 @@
       </c>
       <c r="Q282" s="4" t="n"/>
       <c r="R282" s="4" t="n"/>
+      <c r="S282" s="4" t="inlineStr"/>
+      <c r="T282" s="4" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
@@ -16814,6 +17445,8 @@
       </c>
       <c r="Q283" s="4" t="n"/>
       <c r="R283" s="4" t="n"/>
+      <c r="S283" s="4" t="inlineStr"/>
+      <c r="T283" s="4" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
@@ -16878,6 +17511,8 @@
       </c>
       <c r="Q284" s="4" t="n"/>
       <c r="R284" s="4" t="n"/>
+      <c r="S284" s="4" t="inlineStr"/>
+      <c r="T284" s="4" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
@@ -16942,6 +17577,8 @@
       </c>
       <c r="Q285" s="4" t="n"/>
       <c r="R285" s="4" t="n"/>
+      <c r="S285" s="4" t="inlineStr"/>
+      <c r="T285" s="4" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
@@ -17006,6 +17643,8 @@
       </c>
       <c r="Q286" s="4" t="n"/>
       <c r="R286" s="4" t="n"/>
+      <c r="S286" s="4" t="inlineStr"/>
+      <c r="T286" s="4" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
@@ -17056,6 +17695,8 @@
       <c r="P287" s="4" t="n"/>
       <c r="Q287" s="4" t="n"/>
       <c r="R287" s="4" t="n"/>
+      <c r="S287" s="4" t="inlineStr"/>
+      <c r="T287" s="4" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
@@ -17106,6 +17747,8 @@
       <c r="P288" s="4" t="n"/>
       <c r="Q288" s="4" t="n"/>
       <c r="R288" s="4" t="n"/>
+      <c r="S288" s="4" t="inlineStr"/>
+      <c r="T288" s="4" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
@@ -17156,6 +17799,8 @@
       <c r="P289" s="4" t="n"/>
       <c r="Q289" s="4" t="n"/>
       <c r="R289" s="4" t="n"/>
+      <c r="S289" s="4" t="inlineStr"/>
+      <c r="T289" s="4" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
@@ -17206,6 +17851,8 @@
       <c r="P290" s="4" t="n"/>
       <c r="Q290" s="4" t="n"/>
       <c r="R290" s="4" t="n"/>
+      <c r="S290" s="4" t="inlineStr"/>
+      <c r="T290" s="4" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
@@ -17256,6 +17903,8 @@
       <c r="P291" s="4" t="n"/>
       <c r="Q291" s="4" t="n"/>
       <c r="R291" s="4" t="n"/>
+      <c r="S291" s="4" t="inlineStr"/>
+      <c r="T291" s="4" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
@@ -17306,6 +17955,8 @@
       <c r="P292" s="4" t="n"/>
       <c r="Q292" s="4" t="n"/>
       <c r="R292" s="4" t="n"/>
+      <c r="S292" s="4" t="inlineStr"/>
+      <c r="T292" s="4" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
@@ -17370,6 +18021,8 @@
       </c>
       <c r="Q293" s="4" t="n"/>
       <c r="R293" s="4" t="n"/>
+      <c r="S293" s="4" t="inlineStr"/>
+      <c r="T293" s="4" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
@@ -17434,6 +18087,8 @@
       </c>
       <c r="Q294" s="4" t="n"/>
       <c r="R294" s="4" t="n"/>
+      <c r="S294" s="4" t="inlineStr"/>
+      <c r="T294" s="4" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
@@ -17498,6 +18153,8 @@
       </c>
       <c r="Q295" s="4" t="n"/>
       <c r="R295" s="4" t="n"/>
+      <c r="S295" s="4" t="inlineStr"/>
+      <c r="T295" s="4" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
@@ -17562,6 +18219,8 @@
       </c>
       <c r="Q296" s="4" t="n"/>
       <c r="R296" s="4" t="n"/>
+      <c r="S296" s="4" t="inlineStr"/>
+      <c r="T296" s="4" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
@@ -17626,6 +18285,8 @@
       </c>
       <c r="Q297" s="4" t="n"/>
       <c r="R297" s="4" t="n"/>
+      <c r="S297" s="4" t="inlineStr"/>
+      <c r="T297" s="4" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
@@ -17690,6 +18351,8 @@
       </c>
       <c r="Q298" s="4" t="n"/>
       <c r="R298" s="4" t="n"/>
+      <c r="S298" s="4" t="inlineStr"/>
+      <c r="T298" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -17712,6 +18375,255 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AI1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="34" customWidth="1" min="35" max="35"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>FDRA ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Tool name</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Row index</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Row fuel model</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 1</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 2</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 3</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 4</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 5</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Row break 6</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Column index</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Column fuel model</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 1</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 2</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 3</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 4</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 5</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Column break 6</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Row 1 levels</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>Row 2 levels</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>Row 3 levels</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Row 4 levels</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Row 5 levels</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Row 6 levels</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Row 7 levels</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Class 1</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Class 2</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Class 3</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Class 4</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>Class 5</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>Class 6</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>Class 7</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>Days used</t>
+        </is>
+      </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>Adjustments</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="6">
+    <dataValidation sqref="A2:A5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Use an FDRA ID from the FDOP info sheet." type="list">
+      <formula1>=Lists!$A$1:$A$219</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick the index from the list." type="list">
+      <formula1>=Lists!$B$1:$B$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick the index from the list." type="list">
+      <formula1>=Lists!$B$1:$B$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Fuel model V, W, X, Y or Z." type="list">
+      <formula1>=Lists!$C$1:$C$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Fuel model V, W, X, Y or Z." type="list">
+      <formula1>=Lists!$C$1:$C$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:K5000 N2:S5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Number only" error="Breakpoints are numbers (for example 42 or 55.9)." type="decimal" operator="between">
+      <formula1>-1000</formula1>
+      <formula2>100000</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29083,7 +29995,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>